<commit_message>
greyscale base run 10 times without exclusive rule
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/baserun/greyscale_testrun_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/baserun/greyscale_testrun_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="526">
   <si>
     <t>Filename</t>
   </si>
@@ -817,139 +817,142 @@
     <t>0,1,0,0</t>
   </si>
   <si>
+    <t>0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,1,0</t>
+  </si>
+  <si>
+    <t>0,1,1,0</t>
+  </si>
+  <si>
     <t>1,0,0,0</t>
   </si>
   <si>
-    <t>0,0,1,0</t>
-  </si>
-  <si>
-    <t>0,1,1,0</t>
-  </si>
-  <si>
     <t>0.0357,0.2358,0.0450,0.9244</t>
   </si>
   <si>
-    <t>0.0089,0.3556,0.0057,0.9742</t>
-  </si>
-  <si>
-    <t>0.0164,0.1817,0.0115,0.9798</t>
-  </si>
-  <si>
-    <t>0.0134,0.4157,0.0087,0.9452</t>
-  </si>
-  <si>
-    <t>0.0132,0.7241,0.0207,0.7781</t>
-  </si>
-  <si>
-    <t>0.0164,0.8023,0.0290,0.5742</t>
-  </si>
-  <si>
-    <t>0.0276,0.7209,0.0390,0.4838</t>
-  </si>
-  <si>
-    <t>0.0623,0.5569,0.0323,0.4264</t>
-  </si>
-  <si>
-    <t>0.0222,0.5345,0.0217,0.8710</t>
-  </si>
-  <si>
-    <t>0.0186,0.7874,0.0308,0.5872</t>
-  </si>
-  <si>
-    <t>0.0372,0.7385,0.0360,0.3784</t>
-  </si>
-  <si>
-    <t>0.0195,0.7259,0.0317,0.6252</t>
-  </si>
-  <si>
-    <t>0.0811,0.3551,0.1748,0.3788</t>
-  </si>
-  <si>
-    <t>0.0344,0.6465,0.1439,0.2646</t>
+    <t>0.0089,0.3557,0.0057,0.9742</t>
+  </si>
+  <si>
+    <t>0.0164,0.1818,0.0115,0.9798</t>
+  </si>
+  <si>
+    <t>0.0134,0.4159,0.0087,0.9451</t>
+  </si>
+  <si>
+    <t>0.0132,0.7242,0.0207,0.7780</t>
+  </si>
+  <si>
+    <t>0.0164,0.8024,0.0290,0.5739</t>
+  </si>
+  <si>
+    <t>0.0276,0.7210,0.0390,0.4836</t>
+  </si>
+  <si>
+    <t>0.0623,0.5571,0.0323,0.4262</t>
+  </si>
+  <si>
+    <t>0.0222,0.5347,0.0217,0.8710</t>
+  </si>
+  <si>
+    <t>0.0186,0.7875,0.0308,0.5870</t>
+  </si>
+  <si>
+    <t>0.0372,0.7386,0.0360,0.3782</t>
+  </si>
+  <si>
+    <t>0.0195,0.7260,0.0317,0.6251</t>
+  </si>
+  <si>
+    <t>0.0811,0.3552,0.1748,0.3786</t>
+  </si>
+  <si>
+    <t>0.0344,0.6466,0.1439,0.2645</t>
   </si>
   <si>
     <t>0.0761,0.1337,0.5708,0.1160</t>
   </si>
   <si>
-    <t>0.0290,0.2129,0.5389,0.1170</t>
-  </si>
-  <si>
-    <t>0.0686,0.4429,0.0964,0.4740</t>
+    <t>0.0290,0.2130,0.5389,0.1169</t>
+  </si>
+  <si>
+    <t>0.0686,0.4430,0.0964,0.4738</t>
   </si>
   <si>
     <t>0.0069,0.9624,0.0297,0.1460</t>
   </si>
   <si>
-    <t>0.0186,0.8952,0.0398,0.2654</t>
+    <t>0.0186,0.8952,0.0398,0.2653</t>
   </si>
   <si>
     <t>0.0124,0.8911,0.0396,0.4172</t>
   </si>
   <si>
-    <t>0.0229,0.8330,0.0378,0.3943</t>
-  </si>
-  <si>
-    <t>0.0081,0.9633,0.0541,0.0836</t>
-  </si>
-  <si>
-    <t>0.0819,0.1420,0.1488,0.5269</t>
-  </si>
-  <si>
-    <t>0.0383,0.1436,0.2828,0.4801</t>
-  </si>
-  <si>
-    <t>0.0596,0.0181,0.8155,0.0490</t>
-  </si>
-  <si>
-    <t>0.0546,0.1158,0.5099,0.1803</t>
-  </si>
-  <si>
-    <t>0.0623,0.1182,0.4577,0.1578</t>
+    <t>0.0229,0.8331,0.0378,0.3942</t>
+  </si>
+  <si>
+    <t>0.0081,0.9634,0.0541,0.0836</t>
+  </si>
+  <si>
+    <t>0.0819,0.1420,0.1489,0.5267</t>
+  </si>
+  <si>
+    <t>0.0383,0.1435,0.2829,0.4799</t>
+  </si>
+  <si>
+    <t>0.0596,0.0181,0.8156,0.0490</t>
+  </si>
+  <si>
+    <t>0.0546,0.1158,0.5101,0.1802</t>
+  </si>
+  <si>
+    <t>0.0623,0.1182,0.4580,0.1576</t>
   </si>
   <si>
     <t>0.0624,0.0176,0.8489,0.0425</t>
   </si>
   <si>
-    <t>0.0244,0.0096,0.9323,0.0259</t>
-  </si>
-  <si>
-    <t>0.0274,0.7719,0.0480,0.5064</t>
-  </si>
-  <si>
-    <t>0.0419,0.3602,0.0347,0.8709</t>
-  </si>
-  <si>
-    <t>0.0183,0.2368,0.2053,0.4440</t>
+    <t>0.0244,0.0096,0.9324,0.0259</t>
+  </si>
+  <si>
+    <t>0.0274,0.7720,0.0480,0.5063</t>
+  </si>
+  <si>
+    <t>0.0419,0.3604,0.0347,0.8708</t>
+  </si>
+  <si>
+    <t>0.0183,0.2369,0.2054,0.4437</t>
   </si>
   <si>
     <t>0.0187,0.8647,0.0756,0.1880</t>
   </si>
   <si>
-    <t>0.0815,0.3164,0.0314,0.6560</t>
-  </si>
-  <si>
-    <t>0.0703,0.3295,0.0458,0.6196</t>
-  </si>
-  <si>
-    <t>0.0098,0.8757,0.0221,0.5908</t>
+    <t>0.0815,0.3165,0.0314,0.6559</t>
+  </si>
+  <si>
+    <t>0.0703,0.3297,0.0458,0.6193</t>
+  </si>
+  <si>
+    <t>0.0098,0.8758,0.0221,0.5906</t>
   </si>
   <si>
     <t>0.0223,0.8445,0.0458,0.3975</t>
   </si>
   <si>
-    <t>0.0062,0.9109,0.2190,0.0143</t>
+    <t>0.0062,0.9109,0.2191,0.0143</t>
   </si>
   <si>
     <t>0.0020,0.0048,0.9941,0.0012</t>
   </si>
   <si>
-    <t>0.0214,0.0041,0.9756,0.0029</t>
-  </si>
-  <si>
-    <t>0.0497,0.0430,0.0959,0.8311</t>
-  </si>
-  <si>
-    <t>0.0095,0.5396,0.4562,0.0250</t>
+    <t>0.0214,0.0041,0.9757,0.0029</t>
+  </si>
+  <si>
+    <t>0.0497,0.0430,0.0960,0.8309</t>
+  </si>
+  <si>
+    <t>0.0095,0.5396,0.4563,0.0250</t>
   </si>
   <si>
     <t>0.0051,0.9752,0.0672,0.0211</t>
@@ -958,7 +961,7 @@
     <t>0.0100,0.0220,0.9598,0.0067</t>
   </si>
   <si>
-    <t>0.0086,0.6297,0.0095,0.9346</t>
+    <t>0.0086,0.6299,0.0095,0.9346</t>
   </si>
   <si>
     <t>0.0009,0.9967,0.0081,0.0110</t>
@@ -973,43 +976,43 @@
     <t>0.0042,0.0064,0.9887,0.0012</t>
   </si>
   <si>
-    <t>0.0085,0.0361,0.8806,0.0252</t>
-  </si>
-  <si>
-    <t>0.0213,0.0444,0.8505,0.0354</t>
-  </si>
-  <si>
-    <t>0.0786,0.0709,0.4793,0.1444</t>
-  </si>
-  <si>
-    <t>0.0333,0.0450,0.8368,0.0336</t>
-  </si>
-  <si>
-    <t>0.0250,0.0366,0.8328,0.0505</t>
-  </si>
-  <si>
-    <t>0.0318,0.7521,0.0463,0.3995</t>
-  </si>
-  <si>
-    <t>0.0415,0.6510,0.0449,0.4129</t>
-  </si>
-  <si>
-    <t>0.0095,0.6696,0.0135,0.8935</t>
-  </si>
-  <si>
-    <t>0.0190,0.7670,0.0524,0.4220</t>
-  </si>
-  <si>
-    <t>0.0356,0.6635,0.0396,0.4880</t>
-  </si>
-  <si>
-    <t>0.0309,0.6888,0.0402,0.4963</t>
-  </si>
-  <si>
-    <t>0.0310,0.6999,0.0329,0.5194</t>
-  </si>
-  <si>
-    <t>0.0026,0.9690,0.6082,0.0013</t>
+    <t>0.0085,0.0361,0.8807,0.0251</t>
+  </si>
+  <si>
+    <t>0.0213,0.0444,0.8506,0.0354</t>
+  </si>
+  <si>
+    <t>0.0787,0.0709,0.4794,0.1443</t>
+  </si>
+  <si>
+    <t>0.0333,0.0450,0.8369,0.0336</t>
+  </si>
+  <si>
+    <t>0.0250,0.0366,0.8329,0.0505</t>
+  </si>
+  <si>
+    <t>0.0318,0.7521,0.0463,0.3994</t>
+  </si>
+  <si>
+    <t>0.0415,0.6510,0.0449,0.4128</t>
+  </si>
+  <si>
+    <t>0.0095,0.6698,0.0135,0.8935</t>
+  </si>
+  <si>
+    <t>0.0190,0.7671,0.0524,0.4219</t>
+  </si>
+  <si>
+    <t>0.0356,0.6636,0.0397,0.4878</t>
+  </si>
+  <si>
+    <t>0.0309,0.6890,0.0403,0.4961</t>
+  </si>
+  <si>
+    <t>0.0310,0.6999,0.0329,0.5193</t>
+  </si>
+  <si>
+    <t>0.0026,0.9690,0.6084,0.0013</t>
   </si>
   <si>
     <t>0.0022,0.0074,0.9950,0.0002</t>
@@ -1018,7 +1021,7 @@
     <t>0.0055,0.0077,0.9870,0.0015</t>
   </si>
   <si>
-    <t>0.0049,0.7632,0.8671,0.0016</t>
+    <t>0.0049,0.7631,0.8671,0.0016</t>
   </si>
   <si>
     <t>0.0029,0.0175,0.9900,0.0024</t>
@@ -1030,52 +1033,52 @@
     <t>0.0010,0.9964,0.0186,0.0044</t>
   </si>
   <si>
-    <t>0.0302,0.4733,0.0437,0.8036</t>
-  </si>
-  <si>
-    <t>0.0270,0.6953,0.0775,0.5090</t>
-  </si>
-  <si>
-    <t>0.0187,0.7516,0.1184,0.2222</t>
-  </si>
-  <si>
-    <t>0.0060,0.7536,0.7387,0.0046</t>
+    <t>0.0302,0.4734,0.0437,0.8035</t>
+  </si>
+  <si>
+    <t>0.0270,0.6953,0.0775,0.5088</t>
+  </si>
+  <si>
+    <t>0.0187,0.7517,0.1184,0.2222</t>
+  </si>
+  <si>
+    <t>0.0060,0.7537,0.7388,0.0046</t>
   </si>
   <si>
     <t>0.0063,0.3302,0.9283,0.0014</t>
   </si>
   <si>
-    <t>0.0012,0.9958,0.1475,0.0010</t>
-  </si>
-  <si>
-    <t>0.0043,0.8499,0.5786,0.0038</t>
-  </si>
-  <si>
-    <t>0.0126,0.1153,0.0117,0.9851</t>
-  </si>
-  <si>
-    <t>0.0082,0.4709,0.0064,0.9660</t>
-  </si>
-  <si>
-    <t>0.0074,0.3888,0.0051,0.9782</t>
-  </si>
-  <si>
-    <t>0.0233,0.3082,0.0120,0.9416</t>
-  </si>
-  <si>
-    <t>0.0135,0.3477,0.0111,0.9625</t>
-  </si>
-  <si>
-    <t>0.0127,0.3442,0.0086,0.9657</t>
-  </si>
-  <si>
-    <t>0.0054,0.9734,0.1962,0.0064</t>
+    <t>0.0012,0.9958,0.1476,0.0010</t>
+  </si>
+  <si>
+    <t>0.0043,0.8498,0.5788,0.0038</t>
+  </si>
+  <si>
+    <t>0.0126,0.1154,0.0117,0.9851</t>
+  </si>
+  <si>
+    <t>0.0082,0.4712,0.0064,0.9659</t>
+  </si>
+  <si>
+    <t>0.0074,0.3890,0.0051,0.9782</t>
+  </si>
+  <si>
+    <t>0.0233,0.3084,0.0120,0.9415</t>
+  </si>
+  <si>
+    <t>0.0135,0.3479,0.0111,0.9625</t>
+  </si>
+  <si>
+    <t>0.0127,0.3443,0.0086,0.9657</t>
+  </si>
+  <si>
+    <t>0.0054,0.9734,0.1963,0.0064</t>
   </si>
   <si>
     <t>0.0037,0.0453,0.9857,0.0005</t>
   </si>
   <si>
-    <t>0.0096,0.3184,0.8146,0.0064</t>
+    <t>0.0096,0.3184,0.8147,0.0064</t>
   </si>
   <si>
     <t>0.0090,0.0854,0.9497,0.0024</t>
@@ -1087,67 +1090,67 @@
     <t>0.0063,0.9668,0.1132,0.0174</t>
   </si>
   <si>
-    <t>0.0166,0.7649,0.0267,0.6957</t>
-  </si>
-  <si>
-    <t>0.0191,0.8328,0.0364,0.4294</t>
-  </si>
-  <si>
-    <t>0.0823,0.3422,0.0580,0.8147</t>
-  </si>
-  <si>
-    <t>0.0183,0.8642,0.0343,0.3971</t>
-  </si>
-  <si>
-    <t>0.0196,0.8385,0.0313,0.4233</t>
-  </si>
-  <si>
-    <t>0.0575,0.1824,0.0603,0.9280</t>
-  </si>
-  <si>
-    <t>0.0159,0.8133,0.0290,0.5574</t>
-  </si>
-  <si>
-    <t>0.7596,0.0261,0.0909,0.1322</t>
-  </si>
-  <si>
-    <t>0.0148,0.7697,0.0264,0.6712</t>
-  </si>
-  <si>
-    <t>0.0379,0.2868,0.0360,0.9200</t>
-  </si>
-  <si>
-    <t>0.0222,0.7993,0.0347,0.4626</t>
-  </si>
-  <si>
-    <t>0.0234,0.3685,0.0235,0.9239</t>
-  </si>
-  <si>
-    <t>0.0157,0.5679,0.0210,0.8790</t>
-  </si>
-  <si>
-    <t>0.2650,0.0700,0.0777,0.7626</t>
-  </si>
-  <si>
-    <t>0.0160,0.6906,0.0225,0.7910</t>
-  </si>
-  <si>
-    <t>0.0186,0.7801,0.0274,0.5863</t>
+    <t>0.0166,0.7650,0.0267,0.6956</t>
+  </si>
+  <si>
+    <t>0.0191,0.8329,0.0365,0.4292</t>
+  </si>
+  <si>
+    <t>0.0823,0.3423,0.0580,0.8146</t>
+  </si>
+  <si>
+    <t>0.0183,0.8643,0.0343,0.3969</t>
+  </si>
+  <si>
+    <t>0.0196,0.8385,0.0313,0.4231</t>
+  </si>
+  <si>
+    <t>0.0575,0.1825,0.0603,0.9279</t>
+  </si>
+  <si>
+    <t>0.0159,0.8134,0.0290,0.5572</t>
+  </si>
+  <si>
+    <t>0.7596,0.0261,0.0910,0.1322</t>
+  </si>
+  <si>
+    <t>0.0148,0.7698,0.0264,0.6710</t>
+  </si>
+  <si>
+    <t>0.0379,0.2870,0.0360,0.9199</t>
+  </si>
+  <si>
+    <t>0.0222,0.7994,0.0347,0.4623</t>
+  </si>
+  <si>
+    <t>0.0234,0.3686,0.0235,0.9238</t>
+  </si>
+  <si>
+    <t>0.0157,0.5682,0.0210,0.8788</t>
+  </si>
+  <si>
+    <t>0.2651,0.0700,0.0777,0.7626</t>
+  </si>
+  <si>
+    <t>0.0160,0.6907,0.0225,0.7908</t>
+  </si>
+  <si>
+    <t>0.0186,0.7802,0.0274,0.5861</t>
   </si>
   <si>
     <t>0.0325,0.0089,0.9346,0.0136</t>
   </si>
   <si>
-    <t>0.0566,0.1894,0.2481,0.3864</t>
-  </si>
-  <si>
-    <t>0.1354,0.0846,0.2610,0.2932</t>
-  </si>
-  <si>
-    <t>0.0685,0.0979,0.5661,0.1354</t>
-  </si>
-  <si>
-    <t>0.0104,0.9558,0.0281,0.1228</t>
+    <t>0.0566,0.1895,0.2482,0.3862</t>
+  </si>
+  <si>
+    <t>0.1354,0.0846,0.2611,0.2930</t>
+  </si>
+  <si>
+    <t>0.0685,0.0979,0.5662,0.1353</t>
+  </si>
+  <si>
+    <t>0.0104,0.9559,0.0281,0.1227</t>
   </si>
   <si>
     <t>0.0033,0.9801,0.0154,0.1322</t>
@@ -1156,31 +1159,31 @@
     <t>0.0091,0.9363,0.0289,0.3053</t>
   </si>
   <si>
-    <t>0.0122,0.9125,0.0320,0.3146</t>
-  </si>
-  <si>
-    <t>0.0056,0.9706,0.0202,0.1369</t>
+    <t>0.0122,0.9125,0.0320,0.3144</t>
+  </si>
+  <si>
+    <t>0.0056,0.9706,0.0202,0.1368</t>
   </si>
   <si>
     <t>0.0025,0.9898,0.0138,0.0488</t>
   </si>
   <si>
-    <t>0.0207,0.8387,0.0376,0.4226</t>
-  </si>
-  <si>
-    <t>0.0286,0.7718,0.0560,0.4516</t>
-  </si>
-  <si>
-    <t>0.0366,0.1575,0.3894,0.3416</t>
-  </si>
-  <si>
-    <t>0.0353,0.6928,0.0811,0.4656</t>
-  </si>
-  <si>
-    <t>0.0519,0.5323,0.1296,0.4145</t>
-  </si>
-  <si>
-    <t>0.0232,0.3280,0.1083,0.8814</t>
+    <t>0.0207,0.8387,0.0376,0.4225</t>
+  </si>
+  <si>
+    <t>0.0286,0.7719,0.0560,0.4512</t>
+  </si>
+  <si>
+    <t>0.0366,0.1575,0.3894,0.3415</t>
+  </si>
+  <si>
+    <t>0.0353,0.6928,0.0811,0.4654</t>
+  </si>
+  <si>
+    <t>0.0519,0.5323,0.1296,0.4144</t>
+  </si>
+  <si>
+    <t>0.0232,0.3281,0.1083,0.8813</t>
   </si>
   <si>
     <t>0.0008,0.9979,0.0098,0.0038</t>
@@ -1189,49 +1192,49 @@
     <t>0.0006,0.9982,0.0073,0.0050</t>
   </si>
   <si>
-    <t>0.0047,0.9547,0.0153,0.3638</t>
+    <t>0.0047,0.9547,0.0153,0.3636</t>
   </si>
   <si>
     <t>0.0009,0.9958,0.0131,0.0113</t>
   </si>
   <si>
-    <t>0.0117,0.9487,0.0487,0.1028</t>
-  </si>
-  <si>
-    <t>0.0174,0.8411,0.0352,0.5130</t>
-  </si>
-  <si>
-    <t>0.0164,0.8170,0.0280,0.5987</t>
-  </si>
-  <si>
-    <t>0.0330,0.3400,0.0284,0.8818</t>
-  </si>
-  <si>
-    <t>0.0136,0.3112,0.0122,0.9704</t>
-  </si>
-  <si>
-    <t>0.0206,0.6337,0.0280,0.7858</t>
-  </si>
-  <si>
-    <t>0.0160,0.6491,0.0263,0.7919</t>
-  </si>
-  <si>
-    <t>0.3329,0.2404,0.1198,0.4241</t>
-  </si>
-  <si>
-    <t>0.0231,0.3298,0.0240,0.9149</t>
-  </si>
-  <si>
-    <t>0.0266,0.6991,0.0331,0.5896</t>
-  </si>
-  <si>
-    <t>0.0194,0.7165,0.0244,0.6788</t>
+    <t>0.0117,0.9487,0.0487,0.1027</t>
+  </si>
+  <si>
+    <t>0.0174,0.8411,0.0352,0.5128</t>
+  </si>
+  <si>
+    <t>0.0164,0.8171,0.0280,0.5985</t>
+  </si>
+  <si>
+    <t>0.0330,0.3402,0.0284,0.8817</t>
+  </si>
+  <si>
+    <t>0.0136,0.3113,0.0122,0.9704</t>
+  </si>
+  <si>
+    <t>0.0206,0.6338,0.0280,0.7857</t>
+  </si>
+  <si>
+    <t>0.0160,0.6492,0.0263,0.7918</t>
+  </si>
+  <si>
+    <t>0.3329,0.2404,0.1198,0.4240</t>
+  </si>
+  <si>
+    <t>0.0231,0.3299,0.0240,0.9149</t>
+  </si>
+  <si>
+    <t>0.0266,0.6992,0.0331,0.5895</t>
+  </si>
+  <si>
+    <t>0.0194,0.7167,0.0244,0.6786</t>
   </si>
   <si>
     <t>0.0106,0.1660,0.8909,0.0041</t>
   </si>
   <si>
-    <t>0.0073,0.1320,0.9587,0.0018</t>
+    <t>0.0073,0.1319,0.9588,0.0018</t>
   </si>
   <si>
     <t>0.0053,0.1286,0.9697,0.0016</t>
@@ -1240,49 +1243,49 @@
     <t>0.0291,0.0105,0.9635,0.0030</t>
   </si>
   <si>
-    <t>0.0715,0.3381,0.0709,0.6582</t>
-  </si>
-  <si>
-    <t>0.0375,0.6923,0.0784,0.4343</t>
-  </si>
-  <si>
-    <t>0.0267,0.0883,0.2317,0.7146</t>
-  </si>
-  <si>
-    <t>0.0304,0.6313,0.0706,0.5889</t>
-  </si>
-  <si>
-    <t>0.0285,0.2667,0.0123,0.9350</t>
-  </si>
-  <si>
-    <t>0.0029,0.3530,0.0022,0.9933</t>
-  </si>
-  <si>
-    <t>0.0030,0.3114,0.0021,0.9941</t>
-  </si>
-  <si>
-    <t>0.0147,0.3036,0.0101,0.9669</t>
-  </si>
-  <si>
-    <t>0.0057,0.9294,0.2341,0.0220</t>
-  </si>
-  <si>
-    <t>0.0381,0.6556,0.0359,0.5106</t>
-  </si>
-  <si>
-    <t>0.0181,0.8501,0.0327,0.4405</t>
-  </si>
-  <si>
-    <t>0.0226,0.7153,0.0314,0.6097</t>
-  </si>
-  <si>
-    <t>0.0205,0.8393,0.0375,0.3974</t>
-  </si>
-  <si>
-    <t>0.0158,0.4358,0.0195,0.9226</t>
-  </si>
-  <si>
-    <t>0.5989,0.0014,0.2126,0.0104</t>
+    <t>0.0715,0.3381,0.0710,0.6581</t>
+  </si>
+  <si>
+    <t>0.0375,0.6923,0.0784,0.4342</t>
+  </si>
+  <si>
+    <t>0.0267,0.0883,0.2317,0.7145</t>
+  </si>
+  <si>
+    <t>0.0304,0.6314,0.0706,0.5887</t>
+  </si>
+  <si>
+    <t>0.0285,0.2669,0.0123,0.9350</t>
+  </si>
+  <si>
+    <t>0.0029,0.3533,0.0022,0.9932</t>
+  </si>
+  <si>
+    <t>0.0030,0.3115,0.0021,0.9941</t>
+  </si>
+  <si>
+    <t>0.0147,0.3038,0.0101,0.9668</t>
+  </si>
+  <si>
+    <t>0.0057,0.9294,0.2342,0.0220</t>
+  </si>
+  <si>
+    <t>0.0381,0.6557,0.0359,0.5104</t>
+  </si>
+  <si>
+    <t>0.0181,0.8502,0.0327,0.4402</t>
+  </si>
+  <si>
+    <t>0.0226,0.7153,0.0314,0.6096</t>
+  </si>
+  <si>
+    <t>0.0205,0.8394,0.0375,0.3973</t>
+  </si>
+  <si>
+    <t>0.0158,0.4360,0.0195,0.9225</t>
+  </si>
+  <si>
+    <t>0.5990,0.0014,0.2126,0.0104</t>
   </si>
   <si>
     <t>0.9117,0.0064,0.0375,0.0123</t>
@@ -1291,166 +1294,166 @@
     <t>0.0039,0.0001,0.9888,0.0012</t>
   </si>
   <si>
-    <t>0.0550,0.1694,0.0107,0.8852</t>
-  </si>
-  <si>
-    <t>0.0100,0.5350,0.0102,0.9333</t>
-  </si>
-  <si>
-    <t>0.0581,0.4676,0.0429,0.5849</t>
-  </si>
-  <si>
-    <t>0.0236,0.7521,0.0319,0.6245</t>
-  </si>
-  <si>
-    <t>0.0222,0.6613,0.0307,0.7556</t>
-  </si>
-  <si>
-    <t>0.0262,0.7841,0.0409,0.5407</t>
-  </si>
-  <si>
-    <t>0.0362,0.6639,0.0566,0.5613</t>
-  </si>
-  <si>
-    <t>0.0255,0.6597,0.0527,0.6572</t>
-  </si>
-  <si>
-    <t>0.0194,0.7284,0.0306,0.6861</t>
-  </si>
-  <si>
-    <t>0.0439,0.2036,0.0272,0.9477</t>
-  </si>
-  <si>
-    <t>0.0175,0.7086,0.0299,0.6887</t>
-  </si>
-  <si>
-    <t>0.0368,0.6490,0.0289,0.5392</t>
-  </si>
-  <si>
-    <t>0.0192,0.7281,0.0340,0.6371</t>
-  </si>
-  <si>
-    <t>0.0237,0.6957,0.0381,0.6555</t>
-  </si>
-  <si>
-    <t>0.0189,0.7258,0.0358,0.6223</t>
-  </si>
-  <si>
-    <t>0.0435,0.6822,0.0357,0.4062</t>
-  </si>
-  <si>
-    <t>0.0178,0.7272,0.0281,0.7460</t>
-  </si>
-  <si>
-    <t>0.0090,0.8296,0.0173,0.7427</t>
-  </si>
-  <si>
-    <t>0.0230,0.8013,0.0257,0.4642</t>
-  </si>
-  <si>
-    <t>0.0213,0.7269,0.0379,0.6160</t>
-  </si>
-  <si>
-    <t>0.0366,0.7075,0.0290,0.4367</t>
-  </si>
-  <si>
-    <t>0.0203,0.7521,0.0407,0.5415</t>
-  </si>
-  <si>
-    <t>0.0295,0.6952,0.0274,0.5574</t>
-  </si>
-  <si>
-    <t>0.0246,0.7882,0.0402,0.4699</t>
+    <t>0.0550,0.1695,0.0107,0.8850</t>
+  </si>
+  <si>
+    <t>0.0100,0.5352,0.0102,0.9332</t>
+  </si>
+  <si>
+    <t>0.0581,0.4678,0.0429,0.5846</t>
+  </si>
+  <si>
+    <t>0.0236,0.7522,0.0319,0.6243</t>
+  </si>
+  <si>
+    <t>0.0222,0.6614,0.0307,0.7554</t>
+  </si>
+  <si>
+    <t>0.0262,0.7842,0.0409,0.5406</t>
+  </si>
+  <si>
+    <t>0.0362,0.6639,0.0566,0.5612</t>
+  </si>
+  <si>
+    <t>0.0255,0.6599,0.0527,0.6571</t>
+  </si>
+  <si>
+    <t>0.0194,0.7285,0.0307,0.6859</t>
+  </si>
+  <si>
+    <t>0.0439,0.2037,0.0272,0.9477</t>
+  </si>
+  <si>
+    <t>0.0175,0.7087,0.0299,0.6885</t>
+  </si>
+  <si>
+    <t>0.0368,0.6491,0.0290,0.5391</t>
+  </si>
+  <si>
+    <t>0.0192,0.7281,0.0340,0.6370</t>
+  </si>
+  <si>
+    <t>0.0237,0.6958,0.0381,0.6554</t>
+  </si>
+  <si>
+    <t>0.0189,0.7259,0.0358,0.6221</t>
+  </si>
+  <si>
+    <t>0.0435,0.6824,0.0358,0.4060</t>
+  </si>
+  <si>
+    <t>0.0178,0.7273,0.0282,0.7458</t>
+  </si>
+  <si>
+    <t>0.0090,0.8297,0.0173,0.7425</t>
+  </si>
+  <si>
+    <t>0.0230,0.8014,0.0257,0.4639</t>
+  </si>
+  <si>
+    <t>0.0213,0.7269,0.0379,0.6158</t>
+  </si>
+  <si>
+    <t>0.0366,0.7076,0.0290,0.4365</t>
+  </si>
+  <si>
+    <t>0.0203,0.7521,0.0407,0.5413</t>
+  </si>
+  <si>
+    <t>0.0295,0.6954,0.0274,0.5571</t>
+  </si>
+  <si>
+    <t>0.0246,0.7883,0.0402,0.4697</t>
   </si>
   <si>
     <t>0.0157,0.7698,0.1180,0.1743</t>
   </si>
   <si>
-    <t>0.0270,0.7216,0.0595,0.3921</t>
+    <t>0.0270,0.7217,0.0595,0.3919</t>
   </si>
   <si>
     <t>0.0203,0.0228,0.9368,0.0111</t>
   </si>
   <si>
-    <t>0.0061,0.0971,0.5487,0.2085</t>
-  </si>
-  <si>
-    <t>0.0652,0.3418,0.1199,0.4149</t>
-  </si>
-  <si>
-    <t>0.0109,0.0659,0.9106,0.0084</t>
-  </si>
-  <si>
-    <t>0.0310,0.1080,0.6845,0.0537</t>
+    <t>0.0061,0.0971,0.5489,0.2083</t>
+  </si>
+  <si>
+    <t>0.0652,0.3418,0.1199,0.4147</t>
+  </si>
+  <si>
+    <t>0.0108,0.0659,0.9106,0.0084</t>
+  </si>
+  <si>
+    <t>0.0310,0.1080,0.6846,0.0537</t>
   </si>
   <si>
     <t>0.0420,0.0166,0.9302,0.0080</t>
   </si>
   <si>
-    <t>0.0295,0.0812,0.7045,0.0735</t>
-  </si>
-  <si>
-    <t>0.0295,0.4519,0.2162,0.2507</t>
-  </si>
-  <si>
-    <t>0.0756,0.1443,0.4112,0.2803</t>
-  </si>
-  <si>
-    <t>0.0368,0.6953,0.0723,0.5278</t>
-  </si>
-  <si>
-    <t>0.0427,0.5922,0.1864,0.2064</t>
-  </si>
-  <si>
-    <t>0.0411,0.6621,0.1543,0.2046</t>
-  </si>
-  <si>
-    <t>0.0275,0.2544,0.2594,0.4050</t>
-  </si>
-  <si>
-    <t>0.0434,0.6721,0.1188,0.2884</t>
+    <t>0.0295,0.0812,0.7046,0.0735</t>
+  </si>
+  <si>
+    <t>0.0295,0.4519,0.2162,0.2506</t>
+  </si>
+  <si>
+    <t>0.0756,0.1444,0.4112,0.2802</t>
+  </si>
+  <si>
+    <t>0.0368,0.6954,0.0724,0.5276</t>
+  </si>
+  <si>
+    <t>0.0427,0.5922,0.1864,0.2063</t>
+  </si>
+  <si>
+    <t>0.0411,0.6621,0.1543,0.2045</t>
+  </si>
+  <si>
+    <t>0.0275,0.2544,0.2594,0.4049</t>
+  </si>
+  <si>
+    <t>0.0434,0.6721,0.1189,0.2883</t>
   </si>
   <si>
     <t>0.0333,0.5026,0.1717,0.3477</t>
   </si>
   <si>
-    <t>0.0445,0.4484,0.0716,0.8430</t>
-  </si>
-  <si>
-    <t>0.0107,0.8997,0.0248,0.4434</t>
-  </si>
-  <si>
-    <t>0.0138,0.8841,0.0295,0.4211</t>
-  </si>
-  <si>
-    <t>0.0218,0.8114,0.0294,0.4504</t>
-  </si>
-  <si>
-    <t>0.0193,0.8585,0.0335,0.3697</t>
-  </si>
-  <si>
-    <t>0.0254,0.8287,0.0487,0.4329</t>
-  </si>
-  <si>
-    <t>0.0477,0.3427,0.0476,0.8031</t>
-  </si>
-  <si>
-    <t>0.0469,0.3618,0.1497,0.5310</t>
+    <t>0.0445,0.4485,0.0716,0.8429</t>
+  </si>
+  <si>
+    <t>0.0107,0.8998,0.0248,0.4432</t>
+  </si>
+  <si>
+    <t>0.0138,0.8841,0.0295,0.4210</t>
+  </si>
+  <si>
+    <t>0.0218,0.8115,0.0294,0.4502</t>
+  </si>
+  <si>
+    <t>0.0193,0.8586,0.0335,0.3695</t>
+  </si>
+  <si>
+    <t>0.0254,0.8287,0.0487,0.4328</t>
+  </si>
+  <si>
+    <t>0.0477,0.3429,0.0476,0.8030</t>
+  </si>
+  <si>
+    <t>0.0469,0.3619,0.1497,0.5308</t>
   </si>
   <si>
     <t>0.0284,0.1190,0.2484,0.6529</t>
   </si>
   <si>
-    <t>0.0475,0.5199,0.0884,0.5735</t>
-  </si>
-  <si>
-    <t>0.0252,0.2701,0.3063,0.2778</t>
-  </si>
-  <si>
-    <t>0.0257,0.0614,0.3310,0.5255</t>
-  </si>
-  <si>
-    <t>0.0508,0.0435,0.6125,0.1578</t>
+    <t>0.0475,0.5199,0.0884,0.5733</t>
+  </si>
+  <si>
+    <t>0.0252,0.2702,0.3064,0.2777</t>
+  </si>
+  <si>
+    <t>0.0257,0.0614,0.3312,0.5251</t>
+  </si>
+  <si>
+    <t>0.0508,0.0435,0.6127,0.1576</t>
   </si>
   <si>
     <t>0.0080,0.0048,0.9871,0.0013</t>
@@ -1459,37 +1462,37 @@
     <t>0.0230,0.0445,0.8942,0.0114</t>
   </si>
   <si>
-    <t>0.0408,0.7090,0.0431,0.3635</t>
-  </si>
-  <si>
-    <t>0.0179,0.7752,0.0324,0.5702</t>
-  </si>
-  <si>
-    <t>0.0177,0.8081,0.0326,0.5609</t>
-  </si>
-  <si>
-    <t>0.0366,0.3493,0.0312,0.9011</t>
-  </si>
-  <si>
-    <t>0.0211,0.7326,0.0362,0.6084</t>
-  </si>
-  <si>
-    <t>0.0160,0.8137,0.0298,0.5575</t>
-  </si>
-  <si>
-    <t>0.0128,0.7856,0.0223,0.7030</t>
-  </si>
-  <si>
-    <t>0.0345,0.6989,0.0368,0.4626</t>
-  </si>
-  <si>
-    <t>0.0328,0.4397,0.1246,0.4621</t>
-  </si>
-  <si>
-    <t>0.0281,0.7662,0.0753,0.3020</t>
-  </si>
-  <si>
-    <t>0.0196,0.6124,0.0485,0.6934</t>
+    <t>0.0408,0.7090,0.0431,0.3634</t>
+  </si>
+  <si>
+    <t>0.0179,0.7752,0.0324,0.5701</t>
+  </si>
+  <si>
+    <t>0.0177,0.8082,0.0326,0.5608</t>
+  </si>
+  <si>
+    <t>0.0366,0.3495,0.0312,0.9011</t>
+  </si>
+  <si>
+    <t>0.0211,0.7327,0.0362,0.6083</t>
+  </si>
+  <si>
+    <t>0.0160,0.8138,0.0298,0.5574</t>
+  </si>
+  <si>
+    <t>0.0128,0.7857,0.0223,0.7027</t>
+  </si>
+  <si>
+    <t>0.0345,0.6991,0.0368,0.4623</t>
+  </si>
+  <si>
+    <t>0.0328,0.4399,0.1246,0.4619</t>
+  </si>
+  <si>
+    <t>0.0281,0.7662,0.0753,0.3019</t>
+  </si>
+  <si>
+    <t>0.0196,0.6124,0.0486,0.6933</t>
   </si>
   <si>
     <t>0.0090,0.0258,0.9752,0.0026</t>
@@ -1498,7 +1501,7 @@
     <t>0.0098,0.0249,0.9510,0.0065</t>
   </si>
   <si>
-    <t>0.0269,0.1142,0.6786,0.0741</t>
+    <t>0.0269,0.1141,0.6788,0.0741</t>
   </si>
   <si>
     <t>0.0026,0.0040,0.9938,0.0009</t>
@@ -1513,40 +1516,40 @@
     <t>0.0113,0.0119,0.9770,0.0029</t>
   </si>
   <si>
-    <t>0.0333,0.6222,0.1548,0.2483</t>
-  </si>
-  <si>
-    <t>0.0734,0.0955,0.2265,0.5669</t>
-  </si>
-  <si>
-    <t>0.1091,0.1506,0.1784,0.4449</t>
-  </si>
-  <si>
-    <t>0.0882,0.3320,0.0738,0.5638</t>
-  </si>
-  <si>
-    <t>0.0286,0.8219,0.0345,0.3110</t>
-  </si>
-  <si>
-    <t>0.0359,0.4105,0.0313,0.8783</t>
-  </si>
-  <si>
-    <t>0.0160,0.8299,0.0283,0.5249</t>
-  </si>
-  <si>
-    <t>0.0149,0.8262,0.0280,0.5698</t>
-  </si>
-  <si>
-    <t>0.0234,0.7926,0.0269,0.4600</t>
-  </si>
-  <si>
-    <t>0.0158,0.8410,0.0302,0.5139</t>
-  </si>
-  <si>
-    <t>0.0166,0.8440,0.0314,0.4936</t>
-  </si>
-  <si>
-    <t>0.0092,0.8326,0.0160,0.7163</t>
+    <t>0.0333,0.6223,0.1548,0.2482</t>
+  </si>
+  <si>
+    <t>0.0734,0.0955,0.2266,0.5667</t>
+  </si>
+  <si>
+    <t>0.1091,0.1506,0.1785,0.4447</t>
+  </si>
+  <si>
+    <t>0.0882,0.3320,0.0739,0.5636</t>
+  </si>
+  <si>
+    <t>0.0286,0.8220,0.0345,0.3109</t>
+  </si>
+  <si>
+    <t>0.0359,0.4106,0.0313,0.8782</t>
+  </si>
+  <si>
+    <t>0.0160,0.8299,0.0283,0.5247</t>
+  </si>
+  <si>
+    <t>0.0149,0.8263,0.0280,0.5696</t>
+  </si>
+  <si>
+    <t>0.0234,0.7927,0.0269,0.4597</t>
+  </si>
+  <si>
+    <t>0.0158,0.8410,0.0302,0.5137</t>
+  </si>
+  <si>
+    <t>0.0166,0.8441,0.0314,0.4934</t>
+  </si>
+  <si>
+    <t>0.0092,0.8327,0.0160,0.7162</t>
   </si>
   <si>
     <t>0.0271,0.1477,0.8073,0.0120</t>
@@ -1564,19 +1567,19 @@
     <t>0.0301,0.0059,0.9572,0.0101</t>
   </si>
   <si>
-    <t>0.0389,0.1566,0.0189,0.9335</t>
-  </si>
-  <si>
-    <t>0.0433,0.2239,0.1265,0.6049</t>
-  </si>
-  <si>
-    <t>0.0089,0.0325,0.9463,0.0193</t>
-  </si>
-  <si>
-    <t>0.0116,0.2087,0.0112,0.9797</t>
-  </si>
-  <si>
-    <t>0.0037,0.4546,0.0035,0.9875</t>
+    <t>0.0390,0.1568,0.0190,0.9334</t>
+  </si>
+  <si>
+    <t>0.0433,0.2240,0.1266,0.6047</t>
+  </si>
+  <si>
+    <t>0.0089,0.0325,0.9463,0.0192</t>
+  </si>
+  <si>
+    <t>0.0116,0.2088,0.0112,0.9796</t>
+  </si>
+  <si>
+    <t>0.0037,0.4547,0.0035,0.9875</t>
   </si>
   <si>
     <t>0.0117,0.2884,0.0107,0.9737</t>
@@ -1588,7 +1591,7 @@
     <t>0.0026,0.1264,0.0027,0.9972</t>
   </si>
   <si>
-    <t>0.0070,0.2155,0.0076,0.9902</t>
+    <t>0.0070,0.2156,0.0076,0.9902</t>
   </si>
 </sst>
 </file>
@@ -1974,7 +1977,7 @@
         <v>264</v>
       </c>
       <c r="D2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1988,7 +1991,7 @@
         <v>264</v>
       </c>
       <c r="D3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2002,7 +2005,7 @@
         <v>264</v>
       </c>
       <c r="D4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2016,7 +2019,7 @@
         <v>264</v>
       </c>
       <c r="D5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2030,7 +2033,7 @@
         <v>265</v>
       </c>
       <c r="D6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2044,7 +2047,7 @@
         <v>265</v>
       </c>
       <c r="D7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2058,7 +2061,7 @@
         <v>266</v>
       </c>
       <c r="D8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2072,7 +2075,7 @@
         <v>266</v>
       </c>
       <c r="D9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2086,7 +2089,7 @@
         <v>265</v>
       </c>
       <c r="D10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2100,7 +2103,7 @@
         <v>265</v>
       </c>
       <c r="D11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2114,7 +2117,7 @@
         <v>266</v>
       </c>
       <c r="D12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2128,7 +2131,7 @@
         <v>265</v>
       </c>
       <c r="D13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2142,7 +2145,7 @@
         <v>267</v>
       </c>
       <c r="D14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2156,7 +2159,7 @@
         <v>266</v>
       </c>
       <c r="D15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2170,7 +2173,7 @@
         <v>268</v>
       </c>
       <c r="D16" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2184,7 +2187,7 @@
         <v>268</v>
       </c>
       <c r="D17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2198,7 +2201,7 @@
         <v>267</v>
       </c>
       <c r="D18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2212,7 +2215,7 @@
         <v>266</v>
       </c>
       <c r="D19" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2226,7 +2229,7 @@
         <v>266</v>
       </c>
       <c r="D20" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2240,7 +2243,7 @@
         <v>266</v>
       </c>
       <c r="D21" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2254,7 +2257,7 @@
         <v>266</v>
       </c>
       <c r="D22" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2268,7 +2271,7 @@
         <v>266</v>
       </c>
       <c r="D23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2282,7 +2285,7 @@
         <v>264</v>
       </c>
       <c r="D24" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2296,7 +2299,7 @@
         <v>267</v>
       </c>
       <c r="D25" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2310,7 +2313,7 @@
         <v>268</v>
       </c>
       <c r="D26" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2324,7 +2327,7 @@
         <v>268</v>
       </c>
       <c r="D27" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2338,7 +2341,7 @@
         <v>267</v>
       </c>
       <c r="D28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2352,7 +2355,7 @@
         <v>268</v>
       </c>
       <c r="D29" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2366,7 +2369,7 @@
         <v>268</v>
       </c>
       <c r="D30" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2380,7 +2383,7 @@
         <v>265</v>
       </c>
       <c r="D31" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2394,7 +2397,7 @@
         <v>264</v>
       </c>
       <c r="D32" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2408,7 +2411,7 @@
         <v>267</v>
       </c>
       <c r="D33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2422,7 +2425,7 @@
         <v>266</v>
       </c>
       <c r="D34" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2436,7 +2439,7 @@
         <v>264</v>
       </c>
       <c r="D35" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2450,7 +2453,7 @@
         <v>264</v>
       </c>
       <c r="D36" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2464,7 +2467,7 @@
         <v>265</v>
       </c>
       <c r="D37" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2478,7 +2481,7 @@
         <v>266</v>
       </c>
       <c r="D38" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2492,7 +2495,7 @@
         <v>266</v>
       </c>
       <c r="D39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2506,7 +2509,7 @@
         <v>268</v>
       </c>
       <c r="D40" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2520,7 +2523,7 @@
         <v>268</v>
       </c>
       <c r="D41" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2534,7 +2537,7 @@
         <v>264</v>
       </c>
       <c r="D42" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2548,7 +2551,7 @@
         <v>266</v>
       </c>
       <c r="D43" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2562,7 +2565,7 @@
         <v>266</v>
       </c>
       <c r="D44" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2576,7 +2579,7 @@
         <v>268</v>
       </c>
       <c r="D45" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2590,7 +2593,7 @@
         <v>265</v>
       </c>
       <c r="D46" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2604,7 +2607,7 @@
         <v>266</v>
       </c>
       <c r="D47" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2618,7 +2621,7 @@
         <v>266</v>
       </c>
       <c r="D48" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2632,7 +2635,7 @@
         <v>266</v>
       </c>
       <c r="D49" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2646,7 +2649,7 @@
         <v>268</v>
       </c>
       <c r="D50" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2660,7 +2663,7 @@
         <v>268</v>
       </c>
       <c r="D51" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2674,7 +2677,7 @@
         <v>268</v>
       </c>
       <c r="D52" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2688,7 +2691,7 @@
         <v>267</v>
       </c>
       <c r="D53" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2702,7 +2705,7 @@
         <v>268</v>
       </c>
       <c r="D54" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2716,7 +2719,7 @@
         <v>268</v>
       </c>
       <c r="D55" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2730,7 +2733,7 @@
         <v>266</v>
       </c>
       <c r="D56" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2744,7 +2747,7 @@
         <v>266</v>
       </c>
       <c r="D57" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2758,7 +2761,7 @@
         <v>265</v>
       </c>
       <c r="D58" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2772,7 +2775,7 @@
         <v>266</v>
       </c>
       <c r="D59" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2786,7 +2789,7 @@
         <v>266</v>
       </c>
       <c r="D60" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2800,7 +2803,7 @@
         <v>266</v>
       </c>
       <c r="D61" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -2814,7 +2817,7 @@
         <v>265</v>
       </c>
       <c r="D62" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2828,7 +2831,7 @@
         <v>269</v>
       </c>
       <c r="D63" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2842,7 +2845,7 @@
         <v>268</v>
       </c>
       <c r="D64" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2856,7 +2859,7 @@
         <v>268</v>
       </c>
       <c r="D65" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2870,7 +2873,7 @@
         <v>269</v>
       </c>
       <c r="D66" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2884,7 +2887,7 @@
         <v>268</v>
       </c>
       <c r="D67" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2898,7 +2901,7 @@
         <v>266</v>
       </c>
       <c r="D68" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2912,7 +2915,7 @@
         <v>266</v>
       </c>
       <c r="D69" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2926,7 +2929,7 @@
         <v>264</v>
       </c>
       <c r="D70" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2940,7 +2943,7 @@
         <v>265</v>
       </c>
       <c r="D71" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2954,7 +2957,7 @@
         <v>266</v>
       </c>
       <c r="D72" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2968,7 +2971,7 @@
         <v>269</v>
       </c>
       <c r="D73" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2982,7 +2985,7 @@
         <v>268</v>
       </c>
       <c r="D74" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2996,7 +2999,7 @@
         <v>266</v>
       </c>
       <c r="D75" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3010,7 +3013,7 @@
         <v>269</v>
       </c>
       <c r="D76" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3024,7 +3027,7 @@
         <v>264</v>
       </c>
       <c r="D77" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3038,7 +3041,7 @@
         <v>264</v>
       </c>
       <c r="D78" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3052,7 +3055,7 @@
         <v>264</v>
       </c>
       <c r="D79" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3066,7 +3069,7 @@
         <v>264</v>
       </c>
       <c r="D80" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3080,7 +3083,7 @@
         <v>264</v>
       </c>
       <c r="D81" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3094,7 +3097,7 @@
         <v>264</v>
       </c>
       <c r="D82" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3108,7 +3111,7 @@
         <v>266</v>
       </c>
       <c r="D83" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3122,7 +3125,7 @@
         <v>268</v>
       </c>
       <c r="D84" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3136,7 +3139,7 @@
         <v>268</v>
       </c>
       <c r="D85" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3150,7 +3153,7 @@
         <v>268</v>
       </c>
       <c r="D86" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3164,7 +3167,7 @@
         <v>269</v>
       </c>
       <c r="D87" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3178,7 +3181,7 @@
         <v>266</v>
       </c>
       <c r="D88" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3192,7 +3195,7 @@
         <v>265</v>
       </c>
       <c r="D89" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3206,7 +3209,7 @@
         <v>266</v>
       </c>
       <c r="D90" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3220,7 +3223,7 @@
         <v>264</v>
       </c>
       <c r="D91" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3234,7 +3237,7 @@
         <v>266</v>
       </c>
       <c r="D92" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3248,7 +3251,7 @@
         <v>266</v>
       </c>
       <c r="D93" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3262,7 +3265,7 @@
         <v>264</v>
       </c>
       <c r="D94" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3276,7 +3279,7 @@
         <v>265</v>
       </c>
       <c r="D95" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3287,10 +3290,10 @@
         <v>259</v>
       </c>
       <c r="C96" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D96" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3304,7 +3307,7 @@
         <v>265</v>
       </c>
       <c r="D97" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3318,7 +3321,7 @@
         <v>264</v>
       </c>
       <c r="D98" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3332,7 +3335,7 @@
         <v>266</v>
       </c>
       <c r="D99" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3346,7 +3349,7 @@
         <v>264</v>
       </c>
       <c r="D100" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3360,7 +3363,7 @@
         <v>265</v>
       </c>
       <c r="D101" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3374,7 +3377,7 @@
         <v>264</v>
       </c>
       <c r="D102" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3388,7 +3391,7 @@
         <v>265</v>
       </c>
       <c r="D103" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3402,7 +3405,7 @@
         <v>265</v>
       </c>
       <c r="D104" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3416,7 +3419,7 @@
         <v>268</v>
       </c>
       <c r="D105" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3430,7 +3433,7 @@
         <v>267</v>
       </c>
       <c r="D106" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3444,7 +3447,7 @@
         <v>267</v>
       </c>
       <c r="D107" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3458,7 +3461,7 @@
         <v>268</v>
       </c>
       <c r="D108" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3472,7 +3475,7 @@
         <v>266</v>
       </c>
       <c r="D109" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3486,7 +3489,7 @@
         <v>266</v>
       </c>
       <c r="D110" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3500,7 +3503,7 @@
         <v>266</v>
       </c>
       <c r="D111" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3514,7 +3517,7 @@
         <v>266</v>
       </c>
       <c r="D112" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -3528,7 +3531,7 @@
         <v>266</v>
       </c>
       <c r="D113" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -3542,7 +3545,7 @@
         <v>266</v>
       </c>
       <c r="D114" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -3556,7 +3559,7 @@
         <v>266</v>
       </c>
       <c r="D115" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -3570,7 +3573,7 @@
         <v>266</v>
       </c>
       <c r="D116" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -3584,7 +3587,7 @@
         <v>267</v>
       </c>
       <c r="D117" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -3598,7 +3601,7 @@
         <v>266</v>
       </c>
       <c r="D118" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -3612,7 +3615,7 @@
         <v>266</v>
       </c>
       <c r="D119" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -3626,7 +3629,7 @@
         <v>264</v>
       </c>
       <c r="D120" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -3640,7 +3643,7 @@
         <v>266</v>
       </c>
       <c r="D121" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -3654,7 +3657,7 @@
         <v>266</v>
       </c>
       <c r="D122" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -3668,7 +3671,7 @@
         <v>266</v>
       </c>
       <c r="D123" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -3682,7 +3685,7 @@
         <v>266</v>
       </c>
       <c r="D124" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -3696,7 +3699,7 @@
         <v>266</v>
       </c>
       <c r="D125" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -3710,7 +3713,7 @@
         <v>265</v>
       </c>
       <c r="D126" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -3724,7 +3727,7 @@
         <v>265</v>
       </c>
       <c r="D127" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -3738,7 +3741,7 @@
         <v>264</v>
       </c>
       <c r="D128" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -3752,7 +3755,7 @@
         <v>264</v>
       </c>
       <c r="D129" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -3766,7 +3769,7 @@
         <v>265</v>
       </c>
       <c r="D130" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -3780,7 +3783,7 @@
         <v>265</v>
       </c>
       <c r="D131" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -3794,7 +3797,7 @@
         <v>267</v>
       </c>
       <c r="D132" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -3808,7 +3811,7 @@
         <v>264</v>
       </c>
       <c r="D133" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -3822,7 +3825,7 @@
         <v>265</v>
       </c>
       <c r="D134" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -3836,7 +3839,7 @@
         <v>265</v>
       </c>
       <c r="D135" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -3850,7 +3853,7 @@
         <v>268</v>
       </c>
       <c r="D136" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -3864,7 +3867,7 @@
         <v>268</v>
       </c>
       <c r="D137" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -3878,7 +3881,7 @@
         <v>268</v>
       </c>
       <c r="D138" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -3892,7 +3895,7 @@
         <v>268</v>
       </c>
       <c r="D139" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -3906,7 +3909,7 @@
         <v>264</v>
       </c>
       <c r="D140" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -3920,7 +3923,7 @@
         <v>266</v>
       </c>
       <c r="D141" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -3934,7 +3937,7 @@
         <v>264</v>
       </c>
       <c r="D142" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -3948,7 +3951,7 @@
         <v>265</v>
       </c>
       <c r="D143" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -3962,7 +3965,7 @@
         <v>264</v>
       </c>
       <c r="D144" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -3976,7 +3979,7 @@
         <v>264</v>
       </c>
       <c r="D145" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -3990,7 +3993,7 @@
         <v>264</v>
       </c>
       <c r="D146" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4004,7 +4007,7 @@
         <v>264</v>
       </c>
       <c r="D147" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4018,7 +4021,7 @@
         <v>266</v>
       </c>
       <c r="D148" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4032,7 +4035,7 @@
         <v>265</v>
       </c>
       <c r="D149" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4046,7 +4049,7 @@
         <v>266</v>
       </c>
       <c r="D150" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4060,7 +4063,7 @@
         <v>265</v>
       </c>
       <c r="D151" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4074,7 +4077,7 @@
         <v>266</v>
       </c>
       <c r="D152" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4088,7 +4091,7 @@
         <v>264</v>
       </c>
       <c r="D153" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4099,10 +4102,10 @@
         <v>259</v>
       </c>
       <c r="C154" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D154" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4113,10 +4116,10 @@
         <v>259</v>
       </c>
       <c r="C155" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D155" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4130,7 +4133,7 @@
         <v>268</v>
       </c>
       <c r="D156" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4144,7 +4147,7 @@
         <v>264</v>
       </c>
       <c r="D157" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4158,7 +4161,7 @@
         <v>265</v>
       </c>
       <c r="D158" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4172,7 +4175,7 @@
         <v>264</v>
       </c>
       <c r="D159" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4186,7 +4189,7 @@
         <v>265</v>
       </c>
       <c r="D160" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4200,7 +4203,7 @@
         <v>265</v>
       </c>
       <c r="D161" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4214,7 +4217,7 @@
         <v>265</v>
       </c>
       <c r="D162" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4228,7 +4231,7 @@
         <v>265</v>
       </c>
       <c r="D163" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4242,7 +4245,7 @@
         <v>265</v>
       </c>
       <c r="D164" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4256,7 +4259,7 @@
         <v>265</v>
       </c>
       <c r="D165" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4270,7 +4273,7 @@
         <v>264</v>
       </c>
       <c r="D166" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4284,7 +4287,7 @@
         <v>265</v>
       </c>
       <c r="D167" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4298,7 +4301,7 @@
         <v>265</v>
       </c>
       <c r="D168" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4312,7 +4315,7 @@
         <v>265</v>
       </c>
       <c r="D169" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4326,7 +4329,7 @@
         <v>265</v>
       </c>
       <c r="D170" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4340,7 +4343,7 @@
         <v>265</v>
       </c>
       <c r="D171" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4354,7 +4357,7 @@
         <v>266</v>
       </c>
       <c r="D172" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4368,7 +4371,7 @@
         <v>265</v>
       </c>
       <c r="D173" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4382,7 +4385,7 @@
         <v>265</v>
       </c>
       <c r="D174" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4396,7 +4399,7 @@
         <v>266</v>
       </c>
       <c r="D175" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4410,7 +4413,7 @@
         <v>265</v>
       </c>
       <c r="D176" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4424,7 +4427,7 @@
         <v>266</v>
       </c>
       <c r="D177" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4438,7 +4441,7 @@
         <v>265</v>
       </c>
       <c r="D178" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4452,7 +4455,7 @@
         <v>265</v>
       </c>
       <c r="D179" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4466,7 +4469,7 @@
         <v>266</v>
       </c>
       <c r="D180" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4480,7 +4483,7 @@
         <v>266</v>
       </c>
       <c r="D181" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4494,7 +4497,7 @@
         <v>266</v>
       </c>
       <c r="D182" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4508,7 +4511,7 @@
         <v>268</v>
       </c>
       <c r="D183" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4522,7 +4525,7 @@
         <v>268</v>
       </c>
       <c r="D184" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -4536,7 +4539,7 @@
         <v>267</v>
       </c>
       <c r="D185" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -4550,7 +4553,7 @@
         <v>268</v>
       </c>
       <c r="D186" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -4564,7 +4567,7 @@
         <v>268</v>
       </c>
       <c r="D187" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -4578,7 +4581,7 @@
         <v>268</v>
       </c>
       <c r="D188" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -4592,7 +4595,7 @@
         <v>268</v>
       </c>
       <c r="D189" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -4606,7 +4609,7 @@
         <v>267</v>
       </c>
       <c r="D190" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -4620,7 +4623,7 @@
         <v>267</v>
       </c>
       <c r="D191" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -4634,7 +4637,7 @@
         <v>265</v>
       </c>
       <c r="D192" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -4648,7 +4651,7 @@
         <v>266</v>
       </c>
       <c r="D193" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -4662,7 +4665,7 @@
         <v>266</v>
       </c>
       <c r="D194" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -4676,7 +4679,7 @@
         <v>267</v>
       </c>
       <c r="D195" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -4690,7 +4693,7 @@
         <v>266</v>
       </c>
       <c r="D196" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -4704,7 +4707,7 @@
         <v>266</v>
       </c>
       <c r="D197" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -4718,7 +4721,7 @@
         <v>264</v>
       </c>
       <c r="D198" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -4732,7 +4735,7 @@
         <v>266</v>
       </c>
       <c r="D199" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -4746,7 +4749,7 @@
         <v>266</v>
       </c>
       <c r="D200" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -4760,7 +4763,7 @@
         <v>266</v>
       </c>
       <c r="D201" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -4774,7 +4777,7 @@
         <v>266</v>
       </c>
       <c r="D202" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -4788,7 +4791,7 @@
         <v>266</v>
       </c>
       <c r="D203" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -4802,7 +4805,7 @@
         <v>264</v>
       </c>
       <c r="D204" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -4816,7 +4819,7 @@
         <v>264</v>
       </c>
       <c r="D205" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -4830,7 +4833,7 @@
         <v>264</v>
       </c>
       <c r="D206" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -4844,7 +4847,7 @@
         <v>265</v>
       </c>
       <c r="D207" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -4858,7 +4861,7 @@
         <v>267</v>
       </c>
       <c r="D208" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -4872,7 +4875,7 @@
         <v>264</v>
       </c>
       <c r="D209" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -4886,7 +4889,7 @@
         <v>268</v>
       </c>
       <c r="D210" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -4900,7 +4903,7 @@
         <v>268</v>
       </c>
       <c r="D211" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -4914,7 +4917,7 @@
         <v>268</v>
       </c>
       <c r="D212" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -4928,7 +4931,7 @@
         <v>266</v>
       </c>
       <c r="D213" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -4942,7 +4945,7 @@
         <v>265</v>
       </c>
       <c r="D214" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -4956,7 +4959,7 @@
         <v>265</v>
       </c>
       <c r="D215" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -4970,7 +4973,7 @@
         <v>264</v>
       </c>
       <c r="D216" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -4984,7 +4987,7 @@
         <v>265</v>
       </c>
       <c r="D217" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -4998,7 +5001,7 @@
         <v>265</v>
       </c>
       <c r="D218" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5012,7 +5015,7 @@
         <v>265</v>
       </c>
       <c r="D219" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5026,7 +5029,7 @@
         <v>266</v>
       </c>
       <c r="D220" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5040,7 +5043,7 @@
         <v>267</v>
       </c>
       <c r="D221" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5054,7 +5057,7 @@
         <v>266</v>
       </c>
       <c r="D222" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5068,7 +5071,7 @@
         <v>265</v>
       </c>
       <c r="D223" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5082,7 +5085,7 @@
         <v>268</v>
       </c>
       <c r="D224" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5096,7 +5099,7 @@
         <v>268</v>
       </c>
       <c r="D225" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5110,7 +5113,7 @@
         <v>268</v>
       </c>
       <c r="D226" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5124,7 +5127,7 @@
         <v>268</v>
       </c>
       <c r="D227" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5138,7 +5141,7 @@
         <v>268</v>
       </c>
       <c r="D228" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5152,7 +5155,7 @@
         <v>268</v>
       </c>
       <c r="D229" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5166,7 +5169,7 @@
         <v>268</v>
       </c>
       <c r="D230" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5180,7 +5183,7 @@
         <v>266</v>
       </c>
       <c r="D231" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5194,7 +5197,7 @@
         <v>264</v>
       </c>
       <c r="D232" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5208,7 +5211,7 @@
         <v>267</v>
       </c>
       <c r="D233" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5222,7 +5225,7 @@
         <v>264</v>
       </c>
       <c r="D234" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5236,7 +5239,7 @@
         <v>266</v>
       </c>
       <c r="D235" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5250,7 +5253,7 @@
         <v>264</v>
       </c>
       <c r="D236" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5264,7 +5267,7 @@
         <v>265</v>
       </c>
       <c r="D237" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5278,7 +5281,7 @@
         <v>265</v>
       </c>
       <c r="D238" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5292,7 +5295,7 @@
         <v>266</v>
       </c>
       <c r="D239" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5306,7 +5309,7 @@
         <v>265</v>
       </c>
       <c r="D240" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5320,7 +5323,7 @@
         <v>266</v>
       </c>
       <c r="D241" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5334,7 +5337,7 @@
         <v>265</v>
       </c>
       <c r="D242" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5348,7 +5351,7 @@
         <v>268</v>
       </c>
       <c r="D243" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5362,7 +5365,7 @@
         <v>268</v>
       </c>
       <c r="D244" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5376,7 +5379,7 @@
         <v>268</v>
       </c>
       <c r="D245" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5390,7 +5393,7 @@
         <v>268</v>
       </c>
       <c r="D246" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5404,7 +5407,7 @@
         <v>268</v>
       </c>
       <c r="D247" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -5418,7 +5421,7 @@
         <v>264</v>
       </c>
       <c r="D248" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -5432,7 +5435,7 @@
         <v>264</v>
       </c>
       <c r="D249" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -5446,7 +5449,7 @@
         <v>268</v>
       </c>
       <c r="D250" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -5460,7 +5463,7 @@
         <v>264</v>
       </c>
       <c r="D251" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -5474,7 +5477,7 @@
         <v>264</v>
       </c>
       <c r="D252" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -5488,7 +5491,7 @@
         <v>264</v>
       </c>
       <c r="D253" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -5502,7 +5505,7 @@
         <v>264</v>
       </c>
       <c r="D254" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -5516,7 +5519,7 @@
         <v>264</v>
       </c>
       <c r="D255" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -5530,7 +5533,7 @@
         <v>264</v>
       </c>
       <c r="D256" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>